<commit_message>
Verifica settimanale (parziale): 70 duplicati marcati cross-file
Deduplica globale sui 421 file .xlsx (2844 righe). Corretto un bug di
falso positivo nel matching per dominio: marchi multinazionali con
root domain condiviso tra filiali nazionali indipendenti (sgs.com,
atlascopco.com, systemair.com) venivano erroneamente accorpati tra
paesi diversi (es. Malesia vs Croazia/Serbia); aggiunta guardia che
blocca il merge quando le due righe appartengono a paesi diversi.

Il doppio controllo (upgrade stato_verifica) sui file nuovi è ancora
in corso in background; seguirà un secondo commit con gli upgrade e
l'aggiornamento di weekly_verify_state.json / weekly_verify_log.md.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KaU1epvovxEPcBHjxGKYw
</commit_message>
<xml_diff>
--- a/output/2026-09-03_12_Italia_Campania_Utensilerie_e_Macchine_Utensili.xlsx
+++ b/output/2026-09-03_12_Italia_Campania_Utensilerie_e_Macchine_Utensili.xlsx
@@ -1025,7 +1025,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Via Colonnello Gabriele Pepe 30, Napoli. Forniture industriali, antinfortunistica, trasmissioni industriali. Sito web non trovato/verificabile.</t>
+          <t>Via Colonnello Gabriele Pepe 30, Napoli. Forniture industriali, antinfortunistica, trasmissioni industriali. Sito web non trovato/verificabile. [DUPLICATO — vedi anche: 2026-09-03_04_Italia_Campania_Componentistica-Ventilazione-industriale.xlsx]</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Via S. Cosmo Fuori Porta Nolana 99, Napoli. Forniture industriali. Sito web non trovato/verificabile.</t>
+          <t>Via S. Cosmo Fuori Porta Nolana 99, Napoli. Forniture industriali. Sito web non trovato/verificabile. [DUPLICATO — vedi anche: 2026-09-03_04_Italia_Campania_Componentistica-Ventilazione-industriale.xlsx]</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">

</xml_diff>